<commit_message>
agregando modificaciones a casos de pruebas Spotify
</commit_message>
<xml_diff>
--- a/casos_de_prueba/Casos de prueba app Spotify.xlsx
+++ b/casos_de_prueba/Casos de prueba app Spotify.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="162">
   <si>
     <t>ID</t>
   </si>
@@ -88,9 +88,6 @@
     <t>Validar el rechazo cuando las credenciales son incorrectas</t>
   </si>
   <si>
-    <t>email:isabelmorey@gmail.com Contraseña:isabel2026.</t>
-  </si>
-  <si>
     <t>1- Abrir la aplicación, 2- iniciar sesion, 3- iniciar sesion con contrase;a, 4- rellenar campos</t>
   </si>
   <si>
@@ -424,15 +421,6 @@
     <t>CP-23</t>
   </si>
   <si>
-    <t>El segundo usuario añade una cancion a la cola</t>
-  </si>
-  <si>
-    <t>validar que el anfitrion pausa la cancion</t>
-  </si>
-  <si>
-    <t>1- entrar a la sesion jam, 2- reproducir una cancion, 3- verificar que el segundo usuario visualiza lo mismo, 4- el anfitrion pausa la cancion</t>
-  </si>
-  <si>
     <t>CP-24</t>
   </si>
   <si>
@@ -496,9 +484,6 @@
     <t xml:space="preserve">No pasa </t>
   </si>
   <si>
-    <t>CP-27</t>
-  </si>
-  <si>
     <t>Adaptabilidad en diferentes pantallas</t>
   </si>
   <si>
@@ -512,6 +497,9 @@
   </si>
   <si>
     <t>En ambos dispositivos se adapta la app</t>
+  </si>
+  <si>
+    <t>email:isabelmorey@gmail.com   Contraseña:isabel2026.</t>
   </si>
 </sst>
 </file>
@@ -871,13 +859,13 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:M990"/>
+  <dimension ref="A1:M989"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="8.44140625" customWidth="1"/>
     <col min="2" max="3" width="18.33203125" customWidth="1"/>
     <col min="4" max="4" width="16.6640625" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="5" max="5" width="25.21875" customWidth="1"/>
     <col min="6" max="6" width="30.88671875" customWidth="1"/>
     <col min="7" max="8" width="24.88671875" customWidth="1"/>
     <col min="9" max="9" width="20.6640625" customWidth="1"/>
@@ -979,16 +967,16 @@
         <v>15</v>
       </c>
       <c r="E3" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="F3" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="G3" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="H3" s="11" t="s">
         <v>26</v>
-      </c>
-      <c r="H3" s="11" t="s">
-        <v>27</v>
       </c>
       <c r="I3" s="12" t="s">
         <v>19</v>
@@ -1004,104 +992,104 @@
     </row>
     <row r="4" spans="1:13" ht="39.6">
       <c r="A4" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="C4" s="10" t="s">
         <v>29</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>30</v>
       </c>
       <c r="D4" s="10" t="s">
         <v>15</v>
       </c>
       <c r="E4" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="F4" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="G4" s="10" t="s">
+      <c r="H4" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="H4" s="10" t="s">
+      <c r="I4" s="9" t="s">
         <v>33</v>
-      </c>
-      <c r="I4" s="9" t="s">
-        <v>34</v>
       </c>
       <c r="J4" s="9" t="s">
         <v>20</v>
       </c>
       <c r="K4" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="L4" s="10" t="s">
         <v>35</v>
-      </c>
-      <c r="L4" s="10" t="s">
-        <v>36</v>
       </c>
       <c r="M4" s="8"/>
     </row>
     <row r="5" spans="1:13" ht="39.6">
       <c r="A5" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="C5" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="D5" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="E5" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F5" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="E5" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="F5" s="10" t="s">
+      <c r="G5" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="G5" s="10" t="s">
-        <v>42</v>
-      </c>
       <c r="H5" s="11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I5" s="12" t="s">
         <v>19</v>
       </c>
       <c r="J5" s="12" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="K5" s="12" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L5" s="11"/>
       <c r="M5" s="8"/>
     </row>
     <row r="6" spans="1:13" ht="39.6">
       <c r="A6" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="C6" s="10" t="s">
         <v>45</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>46</v>
       </c>
       <c r="D6" s="10" t="s">
         <v>15</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F6" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="G6" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="G6" s="10" t="s">
-        <v>48</v>
-      </c>
       <c r="H6" s="10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I6" s="9" t="s">
         <v>19</v>
@@ -1117,28 +1105,28 @@
     </row>
     <row r="7" spans="1:13" ht="39.6">
       <c r="A7" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="C7" s="11" t="s">
         <v>50</v>
-      </c>
-      <c r="C7" s="11" t="s">
-        <v>51</v>
       </c>
       <c r="D7" s="10" t="s">
         <v>15</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F7" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="G7" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="G7" s="10" t="s">
-        <v>53</v>
-      </c>
       <c r="H7" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I7" s="12" t="s">
         <v>19</v>
@@ -1154,28 +1142,28 @@
     </row>
     <row r="8" spans="1:13" ht="39.6">
       <c r="A8" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B8" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="C8" s="10" t="s">
         <v>55</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>56</v>
       </c>
       <c r="D8" s="10" t="s">
         <v>15</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F8" s="13" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I8" s="9" t="s">
         <v>19</v>
@@ -1191,28 +1179,28 @@
     </row>
     <row r="9" spans="1:13" ht="39.6">
       <c r="A9" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="B9" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="C9" s="11" t="s">
         <v>59</v>
-      </c>
-      <c r="C9" s="11" t="s">
-        <v>60</v>
       </c>
       <c r="D9" s="10" t="s">
         <v>15</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I9" s="12" t="s">
         <v>19</v>
@@ -1228,28 +1216,28 @@
     </row>
     <row r="10" spans="1:13" ht="52.8">
       <c r="A10" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="C10" s="10" t="s">
         <v>63</v>
-      </c>
-      <c r="C10" s="10" t="s">
-        <v>64</v>
       </c>
       <c r="D10" s="10" t="s">
         <v>15</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F10" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="G10" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="G10" s="10" t="s">
-        <v>66</v>
-      </c>
       <c r="H10" s="10" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I10" s="9" t="s">
         <v>19</v>
@@ -1265,31 +1253,31 @@
     </row>
     <row r="11" spans="1:13" ht="52.8">
       <c r="A11" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="B11" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="C11" s="11" t="s">
         <v>68</v>
-      </c>
-      <c r="C11" s="11" t="s">
-        <v>69</v>
       </c>
       <c r="D11" s="10" t="s">
         <v>15</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F11" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="G11" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="G11" s="10" t="s">
+      <c r="H11" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="H11" s="10" t="s">
-        <v>72</v>
-      </c>
       <c r="I11" s="12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="J11" s="12" t="s">
         <v>20</v>
@@ -1298,34 +1286,34 @@
         <v>20</v>
       </c>
       <c r="L11" s="11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M11" s="8"/>
     </row>
     <row r="12" spans="1:13" ht="52.8">
       <c r="A12" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B12" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="C12" s="11" t="s">
         <v>68</v>
-      </c>
-      <c r="C12" s="11" t="s">
-        <v>69</v>
       </c>
       <c r="D12" s="10" t="s">
         <v>15</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F12" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="H12" s="10" t="s">
         <v>75</v>
-      </c>
-      <c r="G12" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="H12" s="10" t="s">
-        <v>76</v>
       </c>
       <c r="I12" s="9" t="s">
         <v>19</v>
@@ -1341,28 +1329,28 @@
     </row>
     <row r="13" spans="1:13" ht="39.6">
       <c r="A13" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="B13" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="C13" s="10" t="s">
         <v>78</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>79</v>
       </c>
       <c r="D13" s="10" t="s">
         <v>15</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F13" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="G13" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="G13" s="10" t="s">
-        <v>81</v>
-      </c>
       <c r="H13" s="10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="I13" s="9" t="s">
         <v>19</v>
@@ -1378,28 +1366,28 @@
     </row>
     <row r="14" spans="1:13" ht="39.6">
       <c r="A14" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="B14" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="B14" s="14" t="s">
+      <c r="C14" s="11" t="s">
         <v>83</v>
-      </c>
-      <c r="C14" s="11" t="s">
-        <v>84</v>
       </c>
       <c r="D14" s="10" t="s">
         <v>15</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F14" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="G14" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="G14" s="10" t="s">
-        <v>81</v>
-      </c>
       <c r="H14" s="10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="I14" s="9" t="s">
         <v>19</v>
@@ -1415,340 +1403,340 @@
     </row>
     <row r="15" spans="1:13" ht="39.6">
       <c r="A15" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="B15" s="14" t="s">
         <v>85</v>
       </c>
-      <c r="B15" s="14" t="s">
+      <c r="C15" s="10" t="s">
         <v>86</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>87</v>
       </c>
       <c r="D15" s="10" t="s">
         <v>15</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F15" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="G15" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="G15" s="10" t="s">
-        <v>89</v>
-      </c>
       <c r="H15" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="I15" s="9" t="s">
         <v>19</v>
       </c>
       <c r="J15" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="K15" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="L15" s="14"/>
       <c r="M15" s="8"/>
     </row>
     <row r="16" spans="1:13" ht="39.6">
       <c r="A16" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="B16" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="B16" s="14" t="s">
+      <c r="C16" s="11" t="s">
         <v>92</v>
-      </c>
-      <c r="C16" s="11" t="s">
-        <v>93</v>
       </c>
       <c r="D16" s="10" t="s">
         <v>15</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F16" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="G16" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="G16" s="10" t="s">
-        <v>95</v>
-      </c>
       <c r="H16" s="10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I16" s="15" t="s">
         <v>19</v>
       </c>
       <c r="J16" s="15" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="K16" s="15" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="L16" s="14"/>
       <c r="M16" s="8"/>
     </row>
     <row r="17" spans="1:13" ht="39.6">
       <c r="A17" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="B17" s="14" t="s">
         <v>96</v>
       </c>
-      <c r="B17" s="14" t="s">
+      <c r="C17" s="10" t="s">
         <v>97</v>
-      </c>
-      <c r="C17" s="10" t="s">
-        <v>98</v>
       </c>
       <c r="D17" s="10" t="s">
         <v>15</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F17" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="G17" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="G17" s="10" t="s">
-        <v>100</v>
-      </c>
       <c r="H17" s="10" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I17" s="15" t="s">
         <v>19</v>
       </c>
       <c r="J17" s="15" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="K17" s="15" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="L17" s="14"/>
       <c r="M17" s="8"/>
     </row>
     <row r="18" spans="1:13" ht="39.6">
       <c r="A18" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="B18" s="14" t="s">
         <v>101</v>
       </c>
-      <c r="B18" s="14" t="s">
+      <c r="C18" s="11" t="s">
         <v>102</v>
-      </c>
-      <c r="C18" s="11" t="s">
-        <v>103</v>
       </c>
       <c r="D18" s="10" t="s">
         <v>15</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F18" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="G18" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="G18" s="10" t="s">
+      <c r="H18" s="10" t="s">
         <v>105</v>
-      </c>
-      <c r="H18" s="10" t="s">
-        <v>106</v>
       </c>
       <c r="I18" s="15" t="s">
         <v>19</v>
       </c>
       <c r="J18" s="15" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="K18" s="15" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="L18" s="14"/>
       <c r="M18" s="8"/>
     </row>
     <row r="19" spans="1:13" ht="39.6">
       <c r="A19" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="B19" s="14" t="s">
         <v>107</v>
       </c>
-      <c r="B19" s="14" t="s">
+      <c r="C19" s="10" t="s">
         <v>108</v>
-      </c>
-      <c r="C19" s="10" t="s">
-        <v>109</v>
       </c>
       <c r="D19" s="10" t="s">
         <v>15</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F19" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="G19" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="G19" s="10" t="s">
+      <c r="H19" s="14" t="s">
         <v>111</v>
       </c>
-      <c r="H19" s="14" t="s">
-        <v>112</v>
-      </c>
       <c r="I19" s="15" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="J19" s="15" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="K19" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L19" s="14"/>
       <c r="M19" s="8"/>
     </row>
     <row r="20" spans="1:13" ht="52.8">
       <c r="A20" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="B20" s="14" t="s">
         <v>113</v>
       </c>
-      <c r="B20" s="14" t="s">
+      <c r="C20" s="11" t="s">
         <v>114</v>
-      </c>
-      <c r="C20" s="11" t="s">
-        <v>115</v>
       </c>
       <c r="D20" s="10" t="s">
         <v>15</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F20" s="14" t="s">
+        <v>115</v>
+      </c>
+      <c r="G20" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="H20" s="14" t="s">
         <v>116</v>
-      </c>
-      <c r="G20" s="10" t="s">
-        <v>111</v>
-      </c>
-      <c r="H20" s="14" t="s">
-        <v>117</v>
       </c>
       <c r="I20" s="15" t="s">
         <v>19</v>
       </c>
       <c r="J20" s="15" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="K20" s="15" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="L20" s="14"/>
       <c r="M20" s="8"/>
     </row>
     <row r="21" spans="1:13" ht="39.6">
       <c r="A21" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="B21" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="B21" s="14" t="s">
+      <c r="C21" s="10" t="s">
         <v>119</v>
-      </c>
-      <c r="C21" s="10" t="s">
-        <v>120</v>
       </c>
       <c r="D21" s="10" t="s">
         <v>15</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F21" s="14" t="s">
+        <v>120</v>
+      </c>
+      <c r="G21" s="10" t="s">
         <v>121</v>
       </c>
-      <c r="G21" s="10" t="s">
+      <c r="H21" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="H21" s="14" t="s">
-        <v>123</v>
-      </c>
       <c r="I21" s="15" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="J21" s="15" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="K21" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L21" s="14"/>
       <c r="M21" s="8"/>
     </row>
     <row r="22" spans="1:13" ht="39.6">
       <c r="A22" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="B22" s="14" t="s">
         <v>124</v>
       </c>
-      <c r="B22" s="14" t="s">
+      <c r="C22" s="10" t="s">
         <v>125</v>
-      </c>
-      <c r="C22" s="10" t="s">
-        <v>126</v>
       </c>
       <c r="D22" s="10" t="s">
         <v>15</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F22" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="G22" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="G22" s="10" t="s">
+      <c r="H22" s="10" t="s">
         <v>128</v>
-      </c>
-      <c r="H22" s="10" t="s">
-        <v>129</v>
       </c>
       <c r="I22" s="15" t="s">
         <v>19</v>
       </c>
       <c r="J22" s="15" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="K22" s="15" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="L22" s="14"/>
       <c r="M22" s="8"/>
     </row>
     <row r="23" spans="1:13" ht="39.6">
       <c r="A23" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="B23" s="14" t="s">
         <v>130</v>
       </c>
-      <c r="B23" s="14" t="s">
+      <c r="C23" s="14" t="s">
         <v>131</v>
-      </c>
-      <c r="C23" s="14" t="s">
-        <v>132</v>
       </c>
       <c r="D23" s="10" t="s">
         <v>15</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F23" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="G23" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="G23" s="10" t="s">
-        <v>134</v>
-      </c>
       <c r="H23" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I23" s="15" t="s">
         <v>19</v>
       </c>
       <c r="J23" s="15" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="K23" s="15" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="L23" s="14"/>
       <c r="M23" s="8"/>
     </row>
-    <row r="24" spans="1:13" ht="66">
+    <row r="24" spans="1:13" ht="39.6">
       <c r="A24" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B24" s="14" t="s">
         <v>136</v>
@@ -1757,89 +1745,99 @@
         <v>137</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>15</v>
+        <v>138</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F24" s="14" t="s">
-        <v>138</v>
-      </c>
-      <c r="G24" s="10"/>
-      <c r="H24" s="14"/>
-      <c r="I24" s="15"/>
-      <c r="J24" s="15"/>
-      <c r="K24" s="15"/>
+        <v>139</v>
+      </c>
+      <c r="G24" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="H24" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="I24" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="J24" s="15" t="s">
+        <v>89</v>
+      </c>
+      <c r="K24" s="15" t="s">
+        <v>89</v>
+      </c>
       <c r="L24" s="14"/>
       <c r="M24" s="8"/>
     </row>
-    <row r="25" spans="1:13" ht="39.6">
+    <row r="25" spans="1:13" ht="52.8">
       <c r="A25" s="9" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C25" s="14" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>142</v>
+        <v>15</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F25" s="14" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G25" s="10" t="s">
-        <v>144</v>
-      </c>
-      <c r="H25" s="10" t="s">
-        <v>144</v>
+        <v>145</v>
+      </c>
+      <c r="H25" s="14" t="s">
+        <v>146</v>
       </c>
       <c r="I25" s="15" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="J25" s="15" t="s">
-        <v>90</v>
+        <v>147</v>
       </c>
       <c r="K25" s="15" t="s">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="L25" s="14"/>
       <c r="M25" s="8"/>
     </row>
     <row r="26" spans="1:13" ht="52.8">
       <c r="A26" s="9" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="B26" s="14" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C26" s="14" t="s">
+        <v>150</v>
+      </c>
+      <c r="D26" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="E26" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F26" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="G26" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="H26" s="14" t="s">
+        <v>154</v>
+      </c>
+      <c r="I26" s="15" t="s">
+        <v>155</v>
+      </c>
+      <c r="J26" s="15" t="s">
         <v>147</v>
-      </c>
-      <c r="D26" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="E26" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="F26" s="14" t="s">
-        <v>148</v>
-      </c>
-      <c r="G26" s="10" t="s">
-        <v>149</v>
-      </c>
-      <c r="H26" s="14" t="s">
-        <v>150</v>
-      </c>
-      <c r="I26" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="J26" s="15" t="s">
-        <v>151</v>
       </c>
       <c r="K26" s="15" t="s">
         <v>20</v>
@@ -1847,83 +1845,57 @@
       <c r="L26" s="14"/>
       <c r="M26" s="8"/>
     </row>
-    <row r="27" spans="1:13" ht="52.8">
+    <row r="27" spans="1:13" ht="39.6">
       <c r="A27" s="9" t="s">
-        <v>152</v>
-      </c>
-      <c r="B27" s="14" t="s">
-        <v>153</v>
-      </c>
-      <c r="C27" s="14" t="s">
-        <v>154</v>
+        <v>148</v>
+      </c>
+      <c r="B27" s="16" t="s">
+        <v>156</v>
+      </c>
+      <c r="C27" s="16" t="s">
+        <v>157</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="F27" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="G27" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="H27" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="F27" s="16" t="s">
         <v>158</v>
       </c>
-      <c r="I27" s="15" t="s">
+      <c r="G27" s="16" t="s">
         <v>159</v>
       </c>
-      <c r="J27" s="15" t="s">
-        <v>151</v>
-      </c>
-      <c r="K27" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="L27" s="14"/>
+      <c r="H27" s="16" t="s">
+        <v>160</v>
+      </c>
+      <c r="I27" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J27" s="17" t="s">
+        <v>147</v>
+      </c>
+      <c r="K27" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="L27" s="16"/>
       <c r="M27" s="8"/>
     </row>
-    <row r="28" spans="1:13" ht="39.6">
-      <c r="A28" s="9" t="s">
-        <v>160</v>
-      </c>
-      <c r="B28" s="16" t="s">
-        <v>161</v>
-      </c>
-      <c r="C28" s="16" t="s">
-        <v>162</v>
-      </c>
-      <c r="D28" s="10" t="s">
-        <v>155</v>
-      </c>
-      <c r="E28" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="F28" s="16" t="s">
-        <v>163</v>
-      </c>
-      <c r="G28" s="16" t="s">
-        <v>164</v>
-      </c>
-      <c r="H28" s="16" t="s">
-        <v>165</v>
-      </c>
-      <c r="I28" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="J28" s="17" t="s">
-        <v>151</v>
-      </c>
-      <c r="K28" s="17" t="s">
-        <v>90</v>
-      </c>
-      <c r="L28" s="16"/>
-      <c r="M28" s="8"/>
+    <row r="28" spans="1:13" ht="13.2">
+      <c r="A28" s="1"/>
+      <c r="B28" s="2"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+      <c r="L28" s="3"/>
     </row>
     <row r="29" spans="1:13" ht="13.2">
       <c r="A29" s="1"/>
-      <c r="B29" s="2"/>
+      <c r="B29" s="3"/>
       <c r="C29" s="3"/>
       <c r="D29" s="3"/>
       <c r="E29" s="3"/>
@@ -2021,7 +1993,6 @@
       <c r="L37" s="3"/>
     </row>
     <row r="38" spans="1:12" ht="13.2">
-      <c r="A38" s="1"/>
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
       <c r="D38" s="3"/>
@@ -11541,16 +11512,6 @@
       <c r="H989" s="3"/>
       <c r="L989" s="3"/>
     </row>
-    <row r="990" spans="2:12" ht="13.2">
-      <c r="B990" s="3"/>
-      <c r="C990" s="3"/>
-      <c r="D990" s="3"/>
-      <c r="E990" s="3"/>
-      <c r="F990" s="3"/>
-      <c r="G990" s="3"/>
-      <c r="H990" s="3"/>
-      <c r="L990" s="3"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>